<commit_message>
Actualuzo historial_predicciones para ver si funciona webhook
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="75">
   <si>
     <t>id_match</t>
   </si>
@@ -199,14 +199,72 @@
   </si>
   <si>
     <t>platense</t>
+  </si>
+  <si>
+    <t>l2pqAyGf</t>
+  </si>
+  <si>
+    <t>sheffield wed</t>
+  </si>
+  <si>
+    <t>norwich</t>
+  </si>
+  <si>
+    <t>Championship</t>
+  </si>
+  <si>
+    <t>3.30</t>
+  </si>
+  <si>
+    <t>2.20</t>
+  </si>
+  <si>
+    <t>dif_prob_mod_bm &gt; -0.1</t>
+  </si>
+  <si>
+    <t>25lm9eV0</t>
+  </si>
+  <si>
+    <t>southampton</t>
+  </si>
+  <si>
+    <t>coventry</t>
+  </si>
+  <si>
+    <t>1.70</t>
+  </si>
+  <si>
+    <t>4.20</t>
+  </si>
+  <si>
+    <t>4.33</t>
+  </si>
+  <si>
+    <t>YTrCHJNK</t>
+  </si>
+  <si>
+    <t>leeds</t>
+  </si>
+  <si>
+    <t>sunderland</t>
+  </si>
+  <si>
+    <t>1.33</t>
+  </si>
+  <si>
+    <t>5.00</t>
+  </si>
+  <si>
+    <t>9.50</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -236,7 +294,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="51">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -469,6 +527,72 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE1F3EA"/>
         <bgColor rgb="FFE1F3EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFECDD"/>
+        <bgColor rgb="FFCFECDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA1D9BE"/>
+        <bgColor rgb="FFA1D9BE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDFF3E9"/>
+        <bgColor rgb="FFDFF3E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9FD9BC"/>
+        <bgColor rgb="FF9FD9BC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9F0E5"/>
+        <bgColor rgb="FFD9F0E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCFEFD"/>
+        <bgColor rgb="FFFCFEFD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF85CEAA"/>
+        <bgColor rgb="FF85CEAA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F9F5"/>
+        <bgColor rgb="FFF0F9F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF91D3B3"/>
+        <bgColor rgb="FF91D3B3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9F6F0"/>
+        <bgColor rgb="FFE9F6F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAF0E5"/>
+        <bgColor rgb="FFDAF0E5"/>
       </patternFill>
     </fill>
   </fills>
@@ -510,7 +634,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="81">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -666,6 +790,93 @@
     </xf>
     <xf borderId="3" fillId="39" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="40" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="13" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="18" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="27" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="41" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="42" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="43" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="44" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="19" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="41" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="27" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="18" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="45" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="3" fillId="46" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="15" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="47" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="48" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="49" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="50" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1433,6 +1644,215 @@
         <v>28</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="52" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="53">
+        <v>45391.65625</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" s="52" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" s="54">
+        <v>0.29</v>
+      </c>
+      <c r="K9" s="54">
+        <v>0.29</v>
+      </c>
+      <c r="L9" s="55">
+        <v>0.43</v>
+      </c>
+      <c r="M9" s="56">
+        <v>0.0606</v>
+      </c>
+      <c r="N9" s="52">
+        <v>2.0</v>
+      </c>
+      <c r="O9" s="57">
+        <v>0.18</v>
+      </c>
+      <c r="P9" s="58">
+        <v>0.27</v>
+      </c>
+      <c r="Q9" s="59">
+        <v>0.55</v>
+      </c>
+      <c r="R9" s="52">
+        <v>2.0</v>
+      </c>
+      <c r="S9" s="60">
+        <v>0.12329812</v>
+      </c>
+      <c r="T9" s="52">
+        <v>0.551869548</v>
+      </c>
+      <c r="U9" s="52">
+        <v>2.2</v>
+      </c>
+      <c r="V9" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="W9" s="62"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="64">
+        <v>45391.65625</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="63" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="65">
+        <v>0.56</v>
+      </c>
+      <c r="K10" s="66">
+        <v>0.23</v>
+      </c>
+      <c r="L10" s="67">
+        <v>0.22</v>
+      </c>
+      <c r="M10" s="68">
+        <v>0.0573</v>
+      </c>
+      <c r="N10" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="O10" s="69">
+        <v>0.55</v>
+      </c>
+      <c r="P10" s="70">
+        <v>0.27</v>
+      </c>
+      <c r="Q10" s="71">
+        <v>0.18</v>
+      </c>
+      <c r="R10" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="S10" s="72">
+        <v>-0.004713291</v>
+      </c>
+      <c r="T10" s="63">
+        <v>0.551654684</v>
+      </c>
+      <c r="U10" s="63">
+        <v>1.7</v>
+      </c>
+      <c r="V10" s="73" t="s">
+        <v>62</v>
+      </c>
+      <c r="W10" s="74">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="64">
+        <v>45391.666666666664</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="63" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="63" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" s="63" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" s="75">
+        <v>0.71</v>
+      </c>
+      <c r="K11" s="76">
+        <v>0.19</v>
+      </c>
+      <c r="L11" s="77">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="68">
+        <v>0.0571</v>
+      </c>
+      <c r="N11" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="O11" s="78">
+        <v>0.64</v>
+      </c>
+      <c r="P11" s="67">
+        <v>0.22</v>
+      </c>
+      <c r="Q11" s="79">
+        <v>0.14</v>
+      </c>
+      <c r="R11" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="S11" s="80">
+        <v>-0.07574779</v>
+      </c>
+      <c r="T11" s="63">
+        <v>0.635489763</v>
+      </c>
+      <c r="U11" s="63">
+        <v>1.33</v>
+      </c>
+      <c r="V11" s="73" t="s">
+        <v>62</v>
+      </c>
+      <c r="W11" s="62"/>
+    </row>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
Actualizo historial_predicciones y dispatch_event.py
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
   <si>
     <t>id_match</t>
   </si>
@@ -256,6 +256,75 @@
   </si>
   <si>
     <t>9.50</t>
+  </si>
+  <si>
+    <t>bX3RMEa0</t>
+  </si>
+  <si>
+    <t>blackburn</t>
+  </si>
+  <si>
+    <t>dif_prob_mod_bm &lt; 0.0</t>
+  </si>
+  <si>
+    <t>6km0uBnR</t>
+  </si>
+  <si>
+    <t>tottenham</t>
+  </si>
+  <si>
+    <t>dif_prob_mod_bm &gt; -0.05</t>
+  </si>
+  <si>
+    <t>YkKnUd7Q</t>
+  </si>
+  <si>
+    <t>birmingham</t>
+  </si>
+  <si>
+    <t>8rBEPGFs</t>
+  </si>
+  <si>
+    <t>bristol city</t>
+  </si>
+  <si>
+    <t>huddersfield</t>
+  </si>
+  <si>
+    <t>IT65JTP7</t>
+  </si>
+  <si>
+    <t>burnley</t>
+  </si>
+  <si>
+    <t>brighton</t>
+  </si>
+  <si>
+    <t>SbldtiXK</t>
+  </si>
+  <si>
+    <t>manchester city</t>
+  </si>
+  <si>
+    <t>luton</t>
+  </si>
+  <si>
+    <t>dU6KzVfr</t>
+  </si>
+  <si>
+    <t>nottingham</t>
+  </si>
+  <si>
+    <t>wolves</t>
+  </si>
+  <si>
+    <t>WC4gMVuk</t>
+  </si>
+  <si>
+    <t>bournemouth</t>
+  </si>
+  <si>
+    <t>manchester utd</t>
   </si>
 </sst>
 </file>
@@ -294,7 +363,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="51">
+  <fills count="66">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -593,6 +662,96 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDAF0E5"/>
         <bgColor rgb="FFDAF0E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8AD0AE"/>
+        <bgColor rgb="FF8AD0AE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCF1E7"/>
+        <bgColor rgb="FFDCF1E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4E1CB"/>
+        <bgColor rgb="FFB4E1CB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC4E7D6"/>
+        <bgColor rgb="FFC4E7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8E2CE"/>
+        <bgColor rgb="FFB8E2CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EEE1"/>
+        <bgColor rgb="FFD4EEE1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFABDDC5"/>
+        <bgColor rgb="FFABDDC5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF8F3"/>
+        <bgColor rgb="FFEDF8F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6BC398"/>
+        <bgColor rgb="FF6BC398"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1FAF6"/>
+        <bgColor rgb="FFF1FAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FDFB"/>
+        <bgColor rgb="FFF8FDFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF72C69D"/>
+        <bgColor rgb="FF72C69D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5EE"/>
+        <bgColor rgb="FFE8F5EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBFDFC"/>
+        <bgColor rgb="FFFBFDFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -634,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="117">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -876,6 +1035,114 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="50" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="46" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="15" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="47" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="51" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="19" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="34" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="12" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="13" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="52" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="53" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="54" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="21" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="29" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="32" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="55" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="56" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="37" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="57" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="40" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="58" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="59" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="22" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="36" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="21" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="55" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="56" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="60" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="61" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="62" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="63" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="64" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="16" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="38" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="65" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1161,6 +1428,8 @@
       <c r="W1" s="10" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
@@ -1300,6 +1569,8 @@
       <c r="W3" s="10">
         <v>1.0</v>
       </c>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
@@ -1439,6 +1710,8 @@
       <c r="W5" s="10">
         <v>1.0</v>
       </c>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
@@ -1712,6 +1985,8 @@
         <v>62</v>
       </c>
       <c r="W9" s="62"/>
+      <c r="X9" s="62"/>
+      <c r="Y9" s="62"/>
     </row>
     <row r="10">
       <c r="A10" s="63" t="s">
@@ -1783,6 +2058,8 @@
       <c r="W10" s="74">
         <v>1.0</v>
       </c>
+      <c r="X10" s="74"/>
+      <c r="Y10" s="74"/>
     </row>
     <row r="11">
       <c r="A11" s="63" t="s">
@@ -1852,6 +2129,552 @@
         <v>62</v>
       </c>
       <c r="W11" s="62"/>
+      <c r="X11" s="62"/>
+      <c r="Y11" s="62"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="53">
+        <v>45395.354166666664</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="52">
+        <v>1.33</v>
+      </c>
+      <c r="H12" s="52">
+        <v>5.0</v>
+      </c>
+      <c r="I12" s="52">
+        <v>10.0</v>
+      </c>
+      <c r="J12" s="81">
+        <v>0.71</v>
+      </c>
+      <c r="K12" s="82">
+        <v>0.19</v>
+      </c>
+      <c r="L12" s="83">
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="56">
+        <v>0.052</v>
+      </c>
+      <c r="N12" s="52">
+        <v>1.0</v>
+      </c>
+      <c r="O12" s="84">
+        <v>0.68</v>
+      </c>
+      <c r="P12" s="85">
+        <v>0.22</v>
+      </c>
+      <c r="Q12" s="83">
+        <v>0.1</v>
+      </c>
+      <c r="R12" s="52">
+        <v>-1.0</v>
+      </c>
+      <c r="S12" s="86">
+        <v>0.04</v>
+      </c>
+      <c r="T12" s="52">
+        <v>0.32</v>
+      </c>
+      <c r="U12" s="52">
+        <v>3.33</v>
+      </c>
+      <c r="V12" s="61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="64">
+        <v>45395.354166666664</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="63" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="63">
+        <v>2.8</v>
+      </c>
+      <c r="H13" s="63">
+        <v>4.0</v>
+      </c>
+      <c r="I13" s="63">
+        <v>2.2</v>
+      </c>
+      <c r="J13" s="87">
+        <v>0.34</v>
+      </c>
+      <c r="K13" s="88">
+        <v>0.24</v>
+      </c>
+      <c r="L13" s="89">
+        <v>0.43</v>
+      </c>
+      <c r="M13" s="68">
+        <v>0.061688312</v>
+      </c>
+      <c r="N13" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O13" s="90">
+        <v>0.21</v>
+      </c>
+      <c r="P13" s="91">
+        <v>0.44</v>
+      </c>
+      <c r="Q13" s="92">
+        <v>0.35</v>
+      </c>
+      <c r="R13" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="S13" s="93">
+        <v>0.207871625</v>
+      </c>
+      <c r="T13" s="63">
+        <v>0.443345631</v>
+      </c>
+      <c r="U13" s="63">
+        <v>4.0</v>
+      </c>
+      <c r="V13" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C14" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="63">
+        <v>3.1</v>
+      </c>
+      <c r="H14" s="63">
+        <v>3.4</v>
+      </c>
+      <c r="I14" s="63">
+        <v>2.25</v>
+      </c>
+      <c r="J14" s="94">
+        <v>0.3</v>
+      </c>
+      <c r="K14" s="95">
+        <v>0.28</v>
+      </c>
+      <c r="L14" s="96">
+        <v>0.42</v>
+      </c>
+      <c r="M14" s="68">
+        <v>0.061</v>
+      </c>
+      <c r="N14" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="O14" s="93">
+        <v>0.32</v>
+      </c>
+      <c r="P14" s="97">
+        <v>0.26</v>
+      </c>
+      <c r="Q14" s="98">
+        <v>0.41</v>
+      </c>
+      <c r="R14" s="63">
+        <v>-2.0</v>
+      </c>
+      <c r="S14" s="99">
+        <v>0.0</v>
+      </c>
+      <c r="T14" s="63">
+        <v>0.59</v>
+      </c>
+      <c r="U14" s="63">
+        <v>1.62</v>
+      </c>
+      <c r="V14" s="73" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C15" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="63" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="63">
+        <v>2.3</v>
+      </c>
+      <c r="H15" s="63">
+        <v>3.2</v>
+      </c>
+      <c r="I15" s="63">
+        <v>3.3</v>
+      </c>
+      <c r="J15" s="98">
+        <v>0.41</v>
+      </c>
+      <c r="K15" s="94">
+        <v>0.3</v>
+      </c>
+      <c r="L15" s="100">
+        <v>0.29</v>
+      </c>
+      <c r="M15" s="68">
+        <v>0.05</v>
+      </c>
+      <c r="N15" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="O15" s="101">
+        <v>0.49</v>
+      </c>
+      <c r="P15" s="97">
+        <v>0.26</v>
+      </c>
+      <c r="Q15" s="97">
+        <v>0.26</v>
+      </c>
+      <c r="R15" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="S15" s="102">
+        <v>0.07</v>
+      </c>
+      <c r="T15" s="63">
+        <v>0.49</v>
+      </c>
+      <c r="U15" s="63">
+        <v>2.3</v>
+      </c>
+      <c r="V15" s="73" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="53">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="52">
+        <v>3.5</v>
+      </c>
+      <c r="H16" s="52">
+        <v>3.75</v>
+      </c>
+      <c r="I16" s="52">
+        <v>2.0</v>
+      </c>
+      <c r="J16" s="58">
+        <v>0.27</v>
+      </c>
+      <c r="K16" s="103">
+        <v>0.25</v>
+      </c>
+      <c r="L16" s="104">
+        <v>0.48</v>
+      </c>
+      <c r="M16" s="56">
+        <v>0.052380952</v>
+      </c>
+      <c r="N16" s="52">
+        <v>0.0</v>
+      </c>
+      <c r="O16" s="105">
+        <v>0.32</v>
+      </c>
+      <c r="P16" s="106">
+        <v>0.42</v>
+      </c>
+      <c r="Q16" s="107">
+        <v>0.26</v>
+      </c>
+      <c r="R16" s="52">
+        <v>0.0</v>
+      </c>
+      <c r="S16" s="103">
+        <v>0.162065436</v>
+      </c>
+      <c r="T16" s="52">
+        <v>0.415459101</v>
+      </c>
+      <c r="U16" s="52">
+        <v>3.75</v>
+      </c>
+      <c r="V16" s="61" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C17" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="63" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="63">
+        <v>1.1</v>
+      </c>
+      <c r="H17" s="63">
+        <v>11.0</v>
+      </c>
+      <c r="I17" s="63">
+        <v>19.0</v>
+      </c>
+      <c r="J17" s="108">
+        <v>0.86</v>
+      </c>
+      <c r="K17" s="109">
+        <v>0.09</v>
+      </c>
+      <c r="L17" s="110">
+        <v>0.05</v>
+      </c>
+      <c r="M17" s="68">
+        <v>0.052631579</v>
+      </c>
+      <c r="N17" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="O17" s="111">
+        <v>0.82</v>
+      </c>
+      <c r="P17" s="112">
+        <v>0.17</v>
+      </c>
+      <c r="Q17" s="99">
+        <v>0.01</v>
+      </c>
+      <c r="R17" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="S17" s="113">
+        <v>-0.047609234</v>
+      </c>
+      <c r="T17" s="63">
+        <v>0.81602713</v>
+      </c>
+      <c r="U17" s="63">
+        <v>1.1</v>
+      </c>
+      <c r="V17" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="63" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C18" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="63">
+        <v>2.1</v>
+      </c>
+      <c r="H18" s="63">
+        <v>3.4</v>
+      </c>
+      <c r="I18" s="63">
+        <v>3.5</v>
+      </c>
+      <c r="J18" s="114">
+        <v>0.45</v>
+      </c>
+      <c r="K18" s="95">
+        <v>0.28</v>
+      </c>
+      <c r="L18" s="70">
+        <v>0.27</v>
+      </c>
+      <c r="M18" s="68">
+        <v>0.056022409</v>
+      </c>
+      <c r="N18" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O18" s="87">
+        <v>0.34</v>
+      </c>
+      <c r="P18" s="91">
+        <v>0.44</v>
+      </c>
+      <c r="Q18" s="67">
+        <v>0.22</v>
+      </c>
+      <c r="R18" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="S18" s="97">
+        <v>0.16603443</v>
+      </c>
+      <c r="T18" s="63">
+        <v>0.444549019</v>
+      </c>
+      <c r="U18" s="63">
+        <v>3.4</v>
+      </c>
+      <c r="V18" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="64">
+        <v>45395.5625</v>
+      </c>
+      <c r="C19" s="63" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="63" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="63">
+        <v>2.3</v>
+      </c>
+      <c r="H19" s="63">
+        <v>4.0</v>
+      </c>
+      <c r="I19" s="63">
+        <v>2.7</v>
+      </c>
+      <c r="J19" s="98">
+        <v>0.41</v>
+      </c>
+      <c r="K19" s="88">
+        <v>0.24</v>
+      </c>
+      <c r="L19" s="92">
+        <v>0.35</v>
+      </c>
+      <c r="M19" s="68">
+        <v>0.055152979</v>
+      </c>
+      <c r="N19" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="O19" s="95">
+        <v>0.28</v>
+      </c>
+      <c r="P19" s="92">
+        <v>0.35</v>
+      </c>
+      <c r="Q19" s="115">
+        <v>0.37</v>
+      </c>
+      <c r="R19" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="S19" s="116">
+        <v>0.019080418</v>
+      </c>
+      <c r="T19" s="63">
+        <v>0.370091483</v>
+      </c>
+      <c r="U19" s="63">
+        <v>2.7</v>
+      </c>
+      <c r="V19" s="73" t="s">
+        <v>80</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Actualizo historial para ver si dispara dispatch.yml
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="86">
   <si>
     <t>id_match</t>
   </si>
@@ -289,42 +289,6 @@
   </si>
   <si>
     <t>huddersfield</t>
-  </si>
-  <si>
-    <t>IT65JTP7</t>
-  </si>
-  <si>
-    <t>burnley</t>
-  </si>
-  <si>
-    <t>brighton</t>
-  </si>
-  <si>
-    <t>SbldtiXK</t>
-  </si>
-  <si>
-    <t>manchester city</t>
-  </si>
-  <si>
-    <t>luton</t>
-  </si>
-  <si>
-    <t>dU6KzVfr</t>
-  </si>
-  <si>
-    <t>nottingham</t>
-  </si>
-  <si>
-    <t>wolves</t>
-  </si>
-  <si>
-    <t>WC4gMVuk</t>
-  </si>
-  <si>
-    <t>bournemouth</t>
-  </si>
-  <si>
-    <t>manchester utd</t>
   </si>
 </sst>
 </file>
@@ -363,7 +327,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="66">
+  <fills count="60">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -716,42 +680,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEDF8F3"/>
         <bgColor rgb="FFEDF8F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6BC398"/>
-        <bgColor rgb="FF6BC398"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1FAF6"/>
-        <bgColor rgb="FFF1FAF6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FDFB"/>
-        <bgColor rgb="FFF8FDFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF72C69D"/>
-        <bgColor rgb="FF72C69D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5EE"/>
-        <bgColor rgb="FFE8F5EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBFDFC"/>
-        <bgColor rgb="FFFBFDFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -793,7 +721,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="103">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1101,48 +1029,6 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="59" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="22" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="36" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="21" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="55" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="56" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="60" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="61" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="62" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="63" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="64" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="16" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="38" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="65" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2404,278 +2290,6 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="52" t="s">
-        <v>86</v>
-      </c>
-      <c r="B16" s="53">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C16" s="52" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="52" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="52">
-        <v>3.5</v>
-      </c>
-      <c r="H16" s="52">
-        <v>3.75</v>
-      </c>
-      <c r="I16" s="52">
-        <v>2.0</v>
-      </c>
-      <c r="J16" s="58">
-        <v>0.27</v>
-      </c>
-      <c r="K16" s="103">
-        <v>0.25</v>
-      </c>
-      <c r="L16" s="104">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="56">
-        <v>0.052380952</v>
-      </c>
-      <c r="N16" s="52">
-        <v>0.0</v>
-      </c>
-      <c r="O16" s="105">
-        <v>0.32</v>
-      </c>
-      <c r="P16" s="106">
-        <v>0.42</v>
-      </c>
-      <c r="Q16" s="107">
-        <v>0.26</v>
-      </c>
-      <c r="R16" s="52">
-        <v>0.0</v>
-      </c>
-      <c r="S16" s="103">
-        <v>0.162065436</v>
-      </c>
-      <c r="T16" s="52">
-        <v>0.415459101</v>
-      </c>
-      <c r="U16" s="52">
-        <v>3.75</v>
-      </c>
-      <c r="V16" s="61" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="63" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="64">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C17" s="63" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" s="63" t="s">
-        <v>91</v>
-      </c>
-      <c r="E17" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="63">
-        <v>1.1</v>
-      </c>
-      <c r="H17" s="63">
-        <v>11.0</v>
-      </c>
-      <c r="I17" s="63">
-        <v>19.0</v>
-      </c>
-      <c r="J17" s="108">
-        <v>0.86</v>
-      </c>
-      <c r="K17" s="109">
-        <v>0.09</v>
-      </c>
-      <c r="L17" s="110">
-        <v>0.05</v>
-      </c>
-      <c r="M17" s="68">
-        <v>0.052631579</v>
-      </c>
-      <c r="N17" s="63">
-        <v>1.0</v>
-      </c>
-      <c r="O17" s="111">
-        <v>0.82</v>
-      </c>
-      <c r="P17" s="112">
-        <v>0.17</v>
-      </c>
-      <c r="Q17" s="99">
-        <v>0.01</v>
-      </c>
-      <c r="R17" s="63">
-        <v>1.0</v>
-      </c>
-      <c r="S17" s="113">
-        <v>-0.047609234</v>
-      </c>
-      <c r="T17" s="63">
-        <v>0.81602713</v>
-      </c>
-      <c r="U17" s="63">
-        <v>1.1</v>
-      </c>
-      <c r="V17" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="63" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="64">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C18" s="63" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="63" t="s">
-        <v>94</v>
-      </c>
-      <c r="E18" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F18" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="63">
-        <v>2.1</v>
-      </c>
-      <c r="H18" s="63">
-        <v>3.4</v>
-      </c>
-      <c r="I18" s="63">
-        <v>3.5</v>
-      </c>
-      <c r="J18" s="114">
-        <v>0.45</v>
-      </c>
-      <c r="K18" s="95">
-        <v>0.28</v>
-      </c>
-      <c r="L18" s="70">
-        <v>0.27</v>
-      </c>
-      <c r="M18" s="68">
-        <v>0.056022409</v>
-      </c>
-      <c r="N18" s="63">
-        <v>0.0</v>
-      </c>
-      <c r="O18" s="87">
-        <v>0.34</v>
-      </c>
-      <c r="P18" s="91">
-        <v>0.44</v>
-      </c>
-      <c r="Q18" s="67">
-        <v>0.22</v>
-      </c>
-      <c r="R18" s="63">
-        <v>0.0</v>
-      </c>
-      <c r="S18" s="97">
-        <v>0.16603443</v>
-      </c>
-      <c r="T18" s="63">
-        <v>0.444549019</v>
-      </c>
-      <c r="U18" s="63">
-        <v>3.4</v>
-      </c>
-      <c r="V18" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="63" t="s">
-        <v>95</v>
-      </c>
-      <c r="B19" s="64">
-        <v>45395.5625</v>
-      </c>
-      <c r="C19" s="63" t="s">
-        <v>96</v>
-      </c>
-      <c r="D19" s="63" t="s">
-        <v>97</v>
-      </c>
-      <c r="E19" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F19" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="63">
-        <v>2.3</v>
-      </c>
-      <c r="H19" s="63">
-        <v>4.0</v>
-      </c>
-      <c r="I19" s="63">
-        <v>2.7</v>
-      </c>
-      <c r="J19" s="98">
-        <v>0.41</v>
-      </c>
-      <c r="K19" s="88">
-        <v>0.24</v>
-      </c>
-      <c r="L19" s="92">
-        <v>0.35</v>
-      </c>
-      <c r="M19" s="68">
-        <v>0.055152979</v>
-      </c>
-      <c r="N19" s="63">
-        <v>2.0</v>
-      </c>
-      <c r="O19" s="95">
-        <v>0.28</v>
-      </c>
-      <c r="P19" s="92">
-        <v>0.35</v>
-      </c>
-      <c r="Q19" s="115">
-        <v>0.37</v>
-      </c>
-      <c r="R19" s="63">
-        <v>2.0</v>
-      </c>
-      <c r="S19" s="116">
-        <v>0.019080418</v>
-      </c>
-      <c r="T19" s="63">
-        <v>0.370091483</v>
-      </c>
-      <c r="U19" s="63">
-        <v>2.7</v>
-      </c>
-      <c r="V19" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
Actualizo historial tras creaer requirements.txt
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
   <si>
     <t>id_match</t>
   </si>
@@ -289,6 +289,42 @@
   </si>
   <si>
     <t>huddersfield</t>
+  </si>
+  <si>
+    <t>IT65JTP7</t>
+  </si>
+  <si>
+    <t>burnley</t>
+  </si>
+  <si>
+    <t>brighton</t>
+  </si>
+  <si>
+    <t>SbldtiXK</t>
+  </si>
+  <si>
+    <t>manchester city</t>
+  </si>
+  <si>
+    <t>luton</t>
+  </si>
+  <si>
+    <t>dU6KzVfr</t>
+  </si>
+  <si>
+    <t>nottingham</t>
+  </si>
+  <si>
+    <t>wolves</t>
+  </si>
+  <si>
+    <t>WC4gMVuk</t>
+  </si>
+  <si>
+    <t>bournemouth</t>
+  </si>
+  <si>
+    <t>manchester utd</t>
   </si>
 </sst>
 </file>
@@ -327,7 +363,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="60">
+  <fills count="66">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -680,6 +716,42 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEDF8F3"/>
         <bgColor rgb="FFEDF8F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6BC398"/>
+        <bgColor rgb="FF6BC398"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1FAF6"/>
+        <bgColor rgb="FFF1FAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FDFB"/>
+        <bgColor rgb="FFF8FDFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF72C69D"/>
+        <bgColor rgb="FF72C69D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5EE"/>
+        <bgColor rgb="FFE8F5EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBFDFC"/>
+        <bgColor rgb="FFFBFDFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -721,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="117">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1029,6 +1101,48 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="59" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="22" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="36" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="21" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="55" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="56" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="60" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="61" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="62" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="63" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="64" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="16" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="38" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="65" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2290,6 +2404,278 @@
         <v>38</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="53">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="52">
+        <v>3.5</v>
+      </c>
+      <c r="H16" s="52">
+        <v>3.75</v>
+      </c>
+      <c r="I16" s="52">
+        <v>2.0</v>
+      </c>
+      <c r="J16" s="58">
+        <v>0.27</v>
+      </c>
+      <c r="K16" s="103">
+        <v>0.25</v>
+      </c>
+      <c r="L16" s="104">
+        <v>0.48</v>
+      </c>
+      <c r="M16" s="56">
+        <v>0.052380952</v>
+      </c>
+      <c r="N16" s="52">
+        <v>0.0</v>
+      </c>
+      <c r="O16" s="105">
+        <v>0.32</v>
+      </c>
+      <c r="P16" s="106">
+        <v>0.42</v>
+      </c>
+      <c r="Q16" s="107">
+        <v>0.26</v>
+      </c>
+      <c r="R16" s="52">
+        <v>0.0</v>
+      </c>
+      <c r="S16" s="103">
+        <v>0.162065436</v>
+      </c>
+      <c r="T16" s="52">
+        <v>0.415459101</v>
+      </c>
+      <c r="U16" s="52">
+        <v>3.75</v>
+      </c>
+      <c r="V16" s="61" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C17" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="63" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="63">
+        <v>1.1</v>
+      </c>
+      <c r="H17" s="63">
+        <v>11.0</v>
+      </c>
+      <c r="I17" s="63">
+        <v>19.0</v>
+      </c>
+      <c r="J17" s="108">
+        <v>0.86</v>
+      </c>
+      <c r="K17" s="109">
+        <v>0.09</v>
+      </c>
+      <c r="L17" s="110">
+        <v>0.05</v>
+      </c>
+      <c r="M17" s="68">
+        <v>0.052631579</v>
+      </c>
+      <c r="N17" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="O17" s="111">
+        <v>0.82</v>
+      </c>
+      <c r="P17" s="112">
+        <v>0.17</v>
+      </c>
+      <c r="Q17" s="99">
+        <v>0.01</v>
+      </c>
+      <c r="R17" s="63">
+        <v>1.0</v>
+      </c>
+      <c r="S17" s="113">
+        <v>-0.047609234</v>
+      </c>
+      <c r="T17" s="63">
+        <v>0.81602713</v>
+      </c>
+      <c r="U17" s="63">
+        <v>1.1</v>
+      </c>
+      <c r="V17" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="63" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="64">
+        <v>45395.458333333336</v>
+      </c>
+      <c r="C18" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="63">
+        <v>2.1</v>
+      </c>
+      <c r="H18" s="63">
+        <v>3.4</v>
+      </c>
+      <c r="I18" s="63">
+        <v>3.5</v>
+      </c>
+      <c r="J18" s="114">
+        <v>0.45</v>
+      </c>
+      <c r="K18" s="95">
+        <v>0.28</v>
+      </c>
+      <c r="L18" s="70">
+        <v>0.27</v>
+      </c>
+      <c r="M18" s="68">
+        <v>0.056022409</v>
+      </c>
+      <c r="N18" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O18" s="87">
+        <v>0.34</v>
+      </c>
+      <c r="P18" s="91">
+        <v>0.44</v>
+      </c>
+      <c r="Q18" s="67">
+        <v>0.22</v>
+      </c>
+      <c r="R18" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="S18" s="97">
+        <v>0.16603443</v>
+      </c>
+      <c r="T18" s="63">
+        <v>0.444549019</v>
+      </c>
+      <c r="U18" s="63">
+        <v>3.4</v>
+      </c>
+      <c r="V18" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="64">
+        <v>45395.5625</v>
+      </c>
+      <c r="C19" s="63" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="63" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="63">
+        <v>2.3</v>
+      </c>
+      <c r="H19" s="63">
+        <v>4.0</v>
+      </c>
+      <c r="I19" s="63">
+        <v>2.7</v>
+      </c>
+      <c r="J19" s="98">
+        <v>0.41</v>
+      </c>
+      <c r="K19" s="88">
+        <v>0.24</v>
+      </c>
+      <c r="L19" s="92">
+        <v>0.35</v>
+      </c>
+      <c r="M19" s="68">
+        <v>0.055152979</v>
+      </c>
+      <c r="N19" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="O19" s="95">
+        <v>0.28</v>
+      </c>
+      <c r="P19" s="92">
+        <v>0.35</v>
+      </c>
+      <c r="Q19" s="115">
+        <v>0.37</v>
+      </c>
+      <c r="R19" s="63">
+        <v>2.0</v>
+      </c>
+      <c r="S19" s="116">
+        <v>0.019080418</v>
+      </c>
+      <c r="T19" s="63">
+        <v>0.370091483</v>
+      </c>
+      <c r="U19" s="63">
+        <v>2.7</v>
+      </c>
+      <c r="V19" s="73" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
Actualizo historial y veo si se actualiza la pagina automaticamente
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="86">
   <si>
     <t>id_match</t>
   </si>
@@ -289,42 +289,6 @@
   </si>
   <si>
     <t>huddersfield</t>
-  </si>
-  <si>
-    <t>IT65JTP7</t>
-  </si>
-  <si>
-    <t>burnley</t>
-  </si>
-  <si>
-    <t>brighton</t>
-  </si>
-  <si>
-    <t>SbldtiXK</t>
-  </si>
-  <si>
-    <t>manchester city</t>
-  </si>
-  <si>
-    <t>luton</t>
-  </si>
-  <si>
-    <t>dU6KzVfr</t>
-  </si>
-  <si>
-    <t>nottingham</t>
-  </si>
-  <si>
-    <t>wolves</t>
-  </si>
-  <si>
-    <t>WC4gMVuk</t>
-  </si>
-  <si>
-    <t>bournemouth</t>
-  </si>
-  <si>
-    <t>manchester utd</t>
   </si>
 </sst>
 </file>
@@ -363,7 +327,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="66">
+  <fills count="60">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -716,42 +680,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEDF8F3"/>
         <bgColor rgb="FFEDF8F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6BC398"/>
-        <bgColor rgb="FF6BC398"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1FAF6"/>
-        <bgColor rgb="FFF1FAF6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FDFB"/>
-        <bgColor rgb="FFF8FDFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF72C69D"/>
-        <bgColor rgb="FF72C69D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5EE"/>
-        <bgColor rgb="FFE8F5EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBFDFC"/>
-        <bgColor rgb="FFFBFDFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -793,7 +721,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="103">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1101,48 +1029,6 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="59" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="22" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="36" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="21" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="55" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="56" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="60" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="61" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="62" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="63" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="9" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="64" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="16" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="38" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="65" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2404,278 +2290,6 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="52" t="s">
-        <v>86</v>
-      </c>
-      <c r="B16" s="53">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C16" s="52" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="52" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="52">
-        <v>3.5</v>
-      </c>
-      <c r="H16" s="52">
-        <v>3.75</v>
-      </c>
-      <c r="I16" s="52">
-        <v>2.0</v>
-      </c>
-      <c r="J16" s="58">
-        <v>0.27</v>
-      </c>
-      <c r="K16" s="103">
-        <v>0.25</v>
-      </c>
-      <c r="L16" s="104">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="56">
-        <v>0.052380952</v>
-      </c>
-      <c r="N16" s="52">
-        <v>0.0</v>
-      </c>
-      <c r="O16" s="105">
-        <v>0.32</v>
-      </c>
-      <c r="P16" s="106">
-        <v>0.42</v>
-      </c>
-      <c r="Q16" s="107">
-        <v>0.26</v>
-      </c>
-      <c r="R16" s="52">
-        <v>0.0</v>
-      </c>
-      <c r="S16" s="103">
-        <v>0.162065436</v>
-      </c>
-      <c r="T16" s="52">
-        <v>0.415459101</v>
-      </c>
-      <c r="U16" s="52">
-        <v>3.75</v>
-      </c>
-      <c r="V16" s="61" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="63" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="64">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C17" s="63" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" s="63" t="s">
-        <v>91</v>
-      </c>
-      <c r="E17" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="63">
-        <v>1.1</v>
-      </c>
-      <c r="H17" s="63">
-        <v>11.0</v>
-      </c>
-      <c r="I17" s="63">
-        <v>19.0</v>
-      </c>
-      <c r="J17" s="108">
-        <v>0.86</v>
-      </c>
-      <c r="K17" s="109">
-        <v>0.09</v>
-      </c>
-      <c r="L17" s="110">
-        <v>0.05</v>
-      </c>
-      <c r="M17" s="68">
-        <v>0.052631579</v>
-      </c>
-      <c r="N17" s="63">
-        <v>1.0</v>
-      </c>
-      <c r="O17" s="111">
-        <v>0.82</v>
-      </c>
-      <c r="P17" s="112">
-        <v>0.17</v>
-      </c>
-      <c r="Q17" s="99">
-        <v>0.01</v>
-      </c>
-      <c r="R17" s="63">
-        <v>1.0</v>
-      </c>
-      <c r="S17" s="113">
-        <v>-0.047609234</v>
-      </c>
-      <c r="T17" s="63">
-        <v>0.81602713</v>
-      </c>
-      <c r="U17" s="63">
-        <v>1.1</v>
-      </c>
-      <c r="V17" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="63" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="64">
-        <v>45395.458333333336</v>
-      </c>
-      <c r="C18" s="63" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="63" t="s">
-        <v>94</v>
-      </c>
-      <c r="E18" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F18" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="63">
-        <v>2.1</v>
-      </c>
-      <c r="H18" s="63">
-        <v>3.4</v>
-      </c>
-      <c r="I18" s="63">
-        <v>3.5</v>
-      </c>
-      <c r="J18" s="114">
-        <v>0.45</v>
-      </c>
-      <c r="K18" s="95">
-        <v>0.28</v>
-      </c>
-      <c r="L18" s="70">
-        <v>0.27</v>
-      </c>
-      <c r="M18" s="68">
-        <v>0.056022409</v>
-      </c>
-      <c r="N18" s="63">
-        <v>0.0</v>
-      </c>
-      <c r="O18" s="87">
-        <v>0.34</v>
-      </c>
-      <c r="P18" s="91">
-        <v>0.44</v>
-      </c>
-      <c r="Q18" s="67">
-        <v>0.22</v>
-      </c>
-      <c r="R18" s="63">
-        <v>0.0</v>
-      </c>
-      <c r="S18" s="97">
-        <v>0.16603443</v>
-      </c>
-      <c r="T18" s="63">
-        <v>0.444549019</v>
-      </c>
-      <c r="U18" s="63">
-        <v>3.4</v>
-      </c>
-      <c r="V18" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="63" t="s">
-        <v>95</v>
-      </c>
-      <c r="B19" s="64">
-        <v>45395.5625</v>
-      </c>
-      <c r="C19" s="63" t="s">
-        <v>96</v>
-      </c>
-      <c r="D19" s="63" t="s">
-        <v>97</v>
-      </c>
-      <c r="E19" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F19" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="63">
-        <v>2.3</v>
-      </c>
-      <c r="H19" s="63">
-        <v>4.0</v>
-      </c>
-      <c r="I19" s="63">
-        <v>2.7</v>
-      </c>
-      <c r="J19" s="98">
-        <v>0.41</v>
-      </c>
-      <c r="K19" s="88">
-        <v>0.24</v>
-      </c>
-      <c r="L19" s="92">
-        <v>0.35</v>
-      </c>
-      <c r="M19" s="68">
-        <v>0.055152979</v>
-      </c>
-      <c r="N19" s="63">
-        <v>2.0</v>
-      </c>
-      <c r="O19" s="95">
-        <v>0.28</v>
-      </c>
-      <c r="P19" s="92">
-        <v>0.35</v>
-      </c>
-      <c r="Q19" s="115">
-        <v>0.37</v>
-      </c>
-      <c r="R19" s="63">
-        <v>2.0</v>
-      </c>
-      <c r="S19" s="116">
-        <v>0.019080418</v>
-      </c>
-      <c r="T19" s="63">
-        <v>0.370091483</v>
-      </c>
-      <c r="U19" s="63">
-        <v>2.7</v>
-      </c>
-      <c r="V19" s="73" t="s">
-        <v>80</v>
-      </c>
-    </row>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
Update predictions with line-ups
</commit_message>
<xml_diff>
--- a/p6_deployment/data/historial_predicciones.xlsx
+++ b/p6_deployment/data/historial_predicciones.xlsx
@@ -2398,20 +2398,20 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>z7pPU9Zc</t>
+          <t>Sx1kytXA</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.0625</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>columbus crew</t>
+          <t>colorado rapids</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>sporting kansas city</t>
+          <t>cf montreal</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2421,85 +2421,85 @@
         <v>1671</v>
       </c>
       <c r="G29" t="n">
-        <v>1.48</v>
+        <v>1.45</v>
       </c>
       <c r="H29" t="n">
-        <v>4.5</v>
+        <v>4.75</v>
       </c>
       <c r="I29" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="J29" t="n">
-        <v>0.6386964914272737</v>
+        <v>0.6543046357615894</v>
       </c>
       <c r="K29" t="n">
-        <v>0.2100601794027478</v>
+        <v>0.1997350993377483</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1512433291699784</v>
+        <v>0.1459602649006622</v>
       </c>
       <c r="M29" t="n">
-        <v>0.0578978978978979</v>
+        <v>0.05402764204942079</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>0.442947785562681</v>
+        <v>0.3128952493758644</v>
       </c>
       <c r="P29" t="n">
-        <v>0.3696567110004065</v>
+        <v>0.5361372692209605</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.1873955034369123</v>
+        <v>0.150967481403175</v>
       </c>
       <c r="R29" t="n">
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>-0.1957487058645927</v>
+        <v>0.3364021698832122</v>
       </c>
       <c r="T29" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U29" t="n">
-        <v>0.1957487058645927</v>
+        <v>0.3364021698832122</v>
       </c>
       <c r="V29" t="n">
-        <v>0.557052214437319</v>
+        <v>0.5361372692209605</v>
       </c>
       <c r="W29" t="n">
-        <v>2.616279069767442</v>
+        <v>4.75</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
         </is>
       </c>
       <c r="Y29" t="n">
-        <v>38.99365501061233</v>
+        <v>37.52960884546724</v>
       </c>
       <c r="Z29" t="n">
-        <v>38.99365501061233</v>
+        <v>37.52960884546724</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>EcqTTTl4</t>
+          <t>2NHGKPBj</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.0625</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>dc united</t>
+          <t>real salt lake</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>houston dynamo</t>
+          <t>los angeles galaxy</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2509,55 +2509,55 @@
         <v>1671</v>
       </c>
       <c r="G30" t="n">
-        <v>2.1</v>
+        <v>1.73</v>
       </c>
       <c r="H30" t="n">
-        <v>3.7</v>
+        <v>4.33</v>
       </c>
       <c r="I30" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>0.449677174325864</v>
+        <v>0.54584017471928</v>
       </c>
       <c r="K30" t="n">
-        <v>0.2552221800227877</v>
+        <v>0.2180839497146315</v>
       </c>
       <c r="L30" t="n">
-        <v>0.2951006456513482</v>
+        <v>0.2360758755660886</v>
       </c>
       <c r="M30" t="n">
-        <v>0.05896074646074645</v>
+        <v>0.05898156429801493</v>
       </c>
       <c r="N30" t="n">
         <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>0.330849415970903</v>
+        <v>0.2957512568246276</v>
       </c>
       <c r="P30" t="n">
-        <v>0.2884875394026187</v>
+        <v>0.2512322781440824</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.3806630446264782</v>
+        <v>0.4530164650312902</v>
       </c>
       <c r="R30" t="n">
         <v>1</v>
       </c>
       <c r="S30" t="n">
-        <v>0.08556239897512991</v>
+        <v>0.2169405894652016</v>
       </c>
       <c r="T30" t="n">
         <v>2</v>
       </c>
       <c r="U30" t="n">
-        <v>0.08556239897512991</v>
+        <v>0.2169405894652016</v>
       </c>
       <c r="V30" t="n">
-        <v>0.3806630446264782</v>
+        <v>0.4530164650312902</v>
       </c>
       <c r="W30" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -2565,29 +2565,29 @@
         </is>
       </c>
       <c r="Y30" t="n">
-        <v>26.64641312385347</v>
+        <v>31.71115255219031</v>
       </c>
       <c r="Z30" t="n">
-        <v>26.64641312385347</v>
+        <v>31.71115255219031</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>tpoLVkKi</t>
+          <t>UT5bq9li</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.10416666666</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>fc cincinnati</t>
+          <t>los angeles fc</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>new england revolution</t>
+          <t>san jose earthquakes</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2597,85 +2597,85 @@
         <v>1671</v>
       </c>
       <c r="G31" t="n">
-        <v>1.55</v>
+        <v>1.36</v>
       </c>
       <c r="H31" t="n">
-        <v>4.33</v>
+        <v>5.25</v>
       </c>
       <c r="I31" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="J31" t="n">
-        <v>0.6098357297414951</v>
+        <v>0.6880733944954128</v>
       </c>
       <c r="K31" t="n">
-        <v>0.2183014736949925</v>
+        <v>0.1782437745740498</v>
       </c>
       <c r="L31" t="n">
-        <v>0.1718627965635123</v>
+        <v>0.1336828309305373</v>
       </c>
       <c r="M31" t="n">
-        <v>0.05792635435785254</v>
+        <v>0.06862745098039214</v>
       </c>
       <c r="N31" t="n">
         <v>1</v>
       </c>
       <c r="O31" t="n">
-        <v>0.5622116073024658</v>
+        <v>0.6288124535672187</v>
       </c>
       <c r="P31" t="n">
-        <v>0.3421246695652593</v>
+        <v>0.3013673527911105</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.09566372313227506</v>
+        <v>0.06982019364167102</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
       </c>
       <c r="S31" t="n">
-        <v>-0.04762412243902936</v>
+        <v>-0.05926094092819412</v>
       </c>
       <c r="T31" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="U31" t="n">
-        <v>-0.04762412243902936</v>
+        <v>0.05926094092819412</v>
       </c>
       <c r="V31" t="n">
-        <v>0.5622116073024658</v>
+        <v>0.3711875464327813</v>
       </c>
       <c r="W31" t="n">
-        <v>1.55</v>
+        <v>3</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
         </is>
       </c>
       <c r="Y31" t="n">
-        <v>39.3548125111726</v>
+        <v>25.98312825029469</v>
       </c>
       <c r="Z31" t="n">
-        <v>39.3548125111726</v>
+        <v>25.98312825029469</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>ln2oxMH4</t>
+          <t>Ma0gz0nH</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.10416666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>new york red bulls</t>
+          <t>portland timbers</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>toronto fc</t>
+          <t>vancouver whitecaps</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2685,85 +2685,85 @@
         <v>1671</v>
       </c>
       <c r="G32" t="n">
-        <v>1.62</v>
+        <v>2.15</v>
       </c>
       <c r="H32" t="n">
-        <v>4.33</v>
+        <v>3.7</v>
       </c>
       <c r="I32" t="n">
-        <v>5</v>
+        <v>3.1</v>
       </c>
       <c r="J32" t="n">
-        <v>0.5888816959792844</v>
+        <v>0.439632042928325</v>
       </c>
       <c r="K32" t="n">
-        <v>0.2203206345234275</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="L32" t="n">
-        <v>0.1907976694972882</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="M32" t="n">
-        <v>0.0482308328343739</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="N32" t="n">
         <v>1</v>
       </c>
       <c r="O32" t="n">
-        <v>0.4064097840638316</v>
+        <v>0.5201066341798269</v>
       </c>
       <c r="P32" t="n">
-        <v>0.406249628466087</v>
+        <v>0.4046451603515387</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.1873405874700815</v>
+        <v>0.07524820546863475</v>
       </c>
       <c r="R32" t="n">
         <v>1</v>
       </c>
       <c r="S32" t="n">
-        <v>-0.1824719119154528</v>
+        <v>0.08047459125150191</v>
       </c>
       <c r="T32" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U32" t="n">
-        <v>0.1824719119154528</v>
+        <v>0.08047459125150191</v>
       </c>
       <c r="V32" t="n">
-        <v>0.5935902159361683</v>
+        <v>0.5201066341798269</v>
       </c>
       <c r="W32" t="n">
-        <v>2.320471596998928</v>
+        <v>2.15</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
         </is>
       </c>
       <c r="Y32" t="n">
-        <v>41.55131511553179</v>
+        <v>36.40746439258788</v>
       </c>
       <c r="Z32" t="n">
-        <v>41.55131511553179</v>
+        <v>36.40746439258788</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>WYwYSm4A</t>
+          <t>8K42rT3c</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.10416666666</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>orlando city</t>
+          <t>seattle sounders</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>chicago fire</t>
+          <t>fc dallas</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2773,72 +2773,72 @@
         <v>1671</v>
       </c>
       <c r="G33" t="n">
-        <v>1.73</v>
+        <v>1.45</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="I33" t="n">
-        <v>4.33</v>
+        <v>7</v>
       </c>
       <c r="J33" t="n">
-        <v>0.54584017471928</v>
+        <v>0.6538661131292164</v>
       </c>
       <c r="K33" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.210690192008303</v>
       </c>
       <c r="L33" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.1354436948624805</v>
       </c>
       <c r="M33" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.05473453749315826</v>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>0.431972689407671</v>
+        <v>0.3745130758574692</v>
       </c>
       <c r="P33" t="n">
-        <v>0.3757237719572734</v>
+        <v>0.4403573203792</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.1923035386350555</v>
+        <v>0.1851296037633309</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
       </c>
       <c r="S33" t="n">
-        <v>-0.113867485311609</v>
+        <v>0.229667128370897</v>
       </c>
       <c r="T33" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U33" t="n">
-        <v>0.113867485311609</v>
+        <v>0.229667128370897</v>
       </c>
       <c r="V33" t="n">
-        <v>0.568027310592329</v>
+        <v>0.4403573203792</v>
       </c>
       <c r="W33" t="n">
-        <v>2.079231692677071</v>
+        <v>4.5</v>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
         </is>
       </c>
       <c r="Y33" t="n">
-        <v>39.76191174146303</v>
+        <v>30.825012426544</v>
       </c>
       <c r="Z33" t="n">
-        <v>39.76191174146303</v>
+        <v>30.825012426544</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>APxxS7JG</t>
+          <t>z7pPU9Zc</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -2846,12 +2846,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>philadelphia union</t>
+          <t>columbus crew</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>charlotte</t>
+          <t>sporting kansas city</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2861,85 +2861,85 @@
         <v>1671</v>
       </c>
       <c r="G34" t="n">
-        <v>1.9</v>
+        <v>1.38</v>
       </c>
       <c r="H34" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="I34" t="n">
-        <v>3.7</v>
+        <v>7.5</v>
       </c>
       <c r="J34" t="n">
-        <v>0.4998268098372012</v>
+        <v>0.6849315068493151</v>
       </c>
       <c r="K34" t="n">
-        <v>0.2435053688950468</v>
+        <v>0.189041095890411</v>
       </c>
       <c r="L34" t="n">
-        <v>0.2566678212677519</v>
+        <v>0.126027397260274</v>
       </c>
       <c r="M34" t="n">
-        <v>0.05299631615421085</v>
+        <v>0.05797101449275366</v>
       </c>
       <c r="N34" t="n">
         <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>0.4352110096174183</v>
+        <v>0.4761392615476333</v>
       </c>
       <c r="P34" t="n">
-        <v>0.4322347323892172</v>
+        <v>0.3071275721315585</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.1325542579933644</v>
+        <v>0.2167331663208083</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
       </c>
       <c r="S34" t="n">
-        <v>-0.06461580021978297</v>
+        <v>-0.2087922453016819</v>
       </c>
       <c r="T34" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U34" t="n">
-        <v>0.06461580021978297</v>
+        <v>-0.2087922453016819</v>
       </c>
       <c r="V34" t="n">
-        <v>0.5647889903825818</v>
+        <v>0.4761392615476333</v>
       </c>
       <c r="W34" t="n">
-        <v>1.898684210526316</v>
+        <v>1.38</v>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y34" t="n">
-        <v>39.53522932678072</v>
+        <v>33.32974830833433</v>
       </c>
       <c r="Z34" t="n">
-        <v>39.53522932678072</v>
+        <v>33.32974830833433</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>4nxtRRYM</t>
+          <t>EcqTTTl4</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>minnesota united</t>
+          <t>dc united</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>austin fc</t>
+          <t>houston dynamo</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2949,85 +2949,85 @@
         <v>1671</v>
       </c>
       <c r="G35" t="n">
-        <v>1.73</v>
+        <v>2.2</v>
       </c>
       <c r="H35" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="I35" t="n">
-        <v>4.33</v>
+        <v>3</v>
       </c>
       <c r="J35" t="n">
-        <v>0.54584017471928</v>
+        <v>0.4295665634674923</v>
       </c>
       <c r="K35" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.2554179566563468</v>
       </c>
       <c r="L35" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.315015479876161</v>
       </c>
       <c r="M35" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.05814905814905802</v>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="n">
-        <v>0.4585357639156413</v>
+        <v>0.1700536136842038</v>
       </c>
       <c r="P35" t="n">
-        <v>0.3362499079698303</v>
+        <v>0.4010800352937268</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.2052143281145281</v>
+        <v>0.4288663510220694</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
       </c>
       <c r="S35" t="n">
-        <v>-0.08730441080363877</v>
+        <v>0.1138508711459084</v>
       </c>
       <c r="T35" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="U35" t="n">
-        <v>0.08730441080363877</v>
+        <v>0.1138508711459084</v>
       </c>
       <c r="V35" t="n">
-        <v>0.5414642360843587</v>
+        <v>0.4288663510220694</v>
       </c>
       <c r="W35" t="n">
-        <v>2.079231692677071</v>
+        <v>3</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y35" t="n">
-        <v>37.90249652590511</v>
+        <v>30.02064457154486</v>
       </c>
       <c r="Z35" t="n">
-        <v>37.90249652590511</v>
+        <v>30.02064457154486</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>IktpQolT</t>
+          <t>tpoLVkKi</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>nashville sc</t>
+          <t>fc cincinnati</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>new york city</t>
+          <t>new england revolution</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -3037,85 +3037,85 @@
         <v>1671</v>
       </c>
       <c r="G36" t="n">
-        <v>2.25</v>
+        <v>1.6</v>
       </c>
       <c r="H36" t="n">
-        <v>3.3</v>
+        <v>4.5</v>
       </c>
       <c r="I36" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="J36" t="n">
-        <v>0.4192972007147112</v>
+        <v>0.5968169761273209</v>
       </c>
       <c r="K36" t="n">
-        <v>0.2858844550327576</v>
+        <v>0.2122015915119363</v>
       </c>
       <c r="L36" t="n">
-        <v>0.2948183442525313</v>
+        <v>0.1909814323607427</v>
       </c>
       <c r="M36" t="n">
-        <v>0.0599747474747474</v>
+        <v>0.04722222222222228</v>
       </c>
       <c r="N36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O36" t="n">
-        <v>0.3762812603021553</v>
+        <v>0.2399392096277449</v>
       </c>
       <c r="P36" t="n">
-        <v>0.3362450625534014</v>
+        <v>0.4835136265925929</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.2874736771444432</v>
+        <v>0.2765471637796623</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
       </c>
       <c r="S36" t="n">
-        <v>-0.04301594041255591</v>
+        <v>0.2713120350806566</v>
       </c>
       <c r="T36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U36" t="n">
-        <v>-0.04301594041255591</v>
+        <v>0.2713120350806566</v>
       </c>
       <c r="V36" t="n">
-        <v>0.3762812603021553</v>
+        <v>0.4835136265925929</v>
       </c>
       <c r="W36" t="n">
-        <v>2.25</v>
+        <v>4.5</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y36" t="n">
-        <v>26.33968822115087</v>
+        <v>33.8459538614815</v>
       </c>
       <c r="Z36" t="n">
-        <v>26.33968822115087</v>
+        <v>33.8459538614815</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>OWICL5dp</t>
+          <t>ln2oxMH4</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>st  louis city</t>
+          <t>new york red bulls</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>atlanta utd</t>
+          <t>toronto fc</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -3125,85 +3125,85 @@
         <v>1671</v>
       </c>
       <c r="G37" t="n">
-        <v>1.85</v>
+        <v>1.57</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>4.33</v>
       </c>
       <c r="I37" t="n">
-        <v>3.8</v>
+        <v>5.25</v>
       </c>
       <c r="J37" t="n">
-        <v>0.5129935875801552</v>
+        <v>0.6018171661844011</v>
       </c>
       <c r="K37" t="n">
-        <v>0.2372595342558218</v>
+        <v>0.2182108431661685</v>
       </c>
       <c r="L37" t="n">
-        <v>0.2497468781640229</v>
+        <v>0.1799719906494304</v>
       </c>
       <c r="M37" t="n">
-        <v>0.05369843527738261</v>
+        <v>0.05836574785251614</v>
       </c>
       <c r="N37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O37" t="n">
-        <v>0.2433648073553128</v>
+        <v>0.4957472790711372</v>
       </c>
       <c r="P37" t="n">
-        <v>0.3403588267448442</v>
+        <v>0.2448591035222365</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.4162763658998431</v>
+        <v>0.2593936174066264</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
       </c>
       <c r="S37" t="n">
-        <v>0.1665294877358202</v>
+        <v>-0.1060698871132638</v>
       </c>
       <c r="T37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U37" t="n">
-        <v>0.1665294877358202</v>
+        <v>-0.1060698871132638</v>
       </c>
       <c r="V37" t="n">
-        <v>0.4162763658998431</v>
+        <v>0.4957472790711372</v>
       </c>
       <c r="W37" t="n">
-        <v>3.8</v>
+        <v>1.57</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y37" t="n">
-        <v>29.13934561298902</v>
+        <v>34.70230953497961</v>
       </c>
       <c r="Z37" t="n">
-        <v>29.13934561298902</v>
+        <v>34.70230953497961</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>Sx1kytXA</t>
+          <t>WYwYSm4A</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45466.0625</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>colorado rapids</t>
+          <t>orlando city</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>cf montreal</t>
+          <t>chicago fire</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -3213,85 +3213,85 @@
         <v>1671</v>
       </c>
       <c r="G38" t="n">
-        <v>1.45</v>
+        <v>1.65</v>
       </c>
       <c r="H38" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I38" t="n">
         <v>4.75</v>
       </c>
-      <c r="I38" t="n">
-        <v>6.5</v>
-      </c>
       <c r="J38" t="n">
-        <v>0.6543046357615894</v>
+        <v>0.5746381507885073</v>
       </c>
       <c r="K38" t="n">
-        <v>0.1997350993377483</v>
+        <v>0.225750702095485</v>
       </c>
       <c r="L38" t="n">
-        <v>0.1459602649006622</v>
+        <v>0.1996111471160078</v>
       </c>
       <c r="M38" t="n">
-        <v>0.05402764204942079</v>
+        <v>0.05468215994531778</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
       </c>
       <c r="O38" t="n">
-        <v>0.3128952493758644</v>
+        <v>0.2064575634094828</v>
       </c>
       <c r="P38" t="n">
-        <v>0.5361372692209605</v>
+        <v>0.4346844708020633</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.150967481403175</v>
+        <v>0.3588579657884538</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
       </c>
       <c r="S38" t="n">
-        <v>0.3364021698832122</v>
+        <v>0.2089337687065784</v>
       </c>
       <c r="T38" t="n">
         <v>0</v>
       </c>
       <c r="U38" t="n">
-        <v>0.3364021698832122</v>
+        <v>0.2089337687065784</v>
       </c>
       <c r="V38" t="n">
-        <v>0.5361372692209605</v>
+        <v>0.4346844708020633</v>
       </c>
       <c r="W38" t="n">
-        <v>4.75</v>
+        <v>4.2</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y38" t="n">
-        <v>37.52960884546724</v>
+        <v>30.42791295614444</v>
       </c>
       <c r="Z38" t="n">
-        <v>37.52960884546724</v>
+        <v>30.42791295614444</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>2NHGKPBj</t>
+          <t>APxxS7JG</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45466.0625</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>real salt lake</t>
+          <t>philadelphia union</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>los angeles galaxy</t>
+          <t>charlotte</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -3301,85 +3301,85 @@
         <v>1671</v>
       </c>
       <c r="G39" t="n">
-        <v>1.73</v>
+        <v>2.25</v>
       </c>
       <c r="H39" t="n">
-        <v>4.33</v>
+        <v>3.7</v>
       </c>
       <c r="I39" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="J39" t="n">
-        <v>0.54584017471928</v>
+        <v>0.4194683346364347</v>
       </c>
       <c r="K39" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.2550820953870211</v>
       </c>
       <c r="L39" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.3254495699765442</v>
       </c>
       <c r="M39" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.05954230092161117</v>
       </c>
       <c r="N39" t="n">
         <v>2</v>
       </c>
       <c r="O39" t="n">
-        <v>0.2957512568246276</v>
+        <v>0.1470755222311179</v>
       </c>
       <c r="P39" t="n">
-        <v>0.2512322781440824</v>
+        <v>0.3804223516987789</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.4530164650312902</v>
+        <v>0.4725021260701033</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
       </c>
       <c r="S39" t="n">
-        <v>0.2169405894652016</v>
+        <v>0.1470525560935591</v>
       </c>
       <c r="T39" t="n">
         <v>2</v>
       </c>
       <c r="U39" t="n">
-        <v>0.2169405894652016</v>
+        <v>0.1470525560935591</v>
       </c>
       <c r="V39" t="n">
-        <v>0.4530164650312902</v>
+        <v>0.4725021260701033</v>
       </c>
       <c r="W39" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y39" t="n">
-        <v>31.71115255219031</v>
+        <v>33.07514882490723</v>
       </c>
       <c r="Z39" t="n">
-        <v>31.71115255219031</v>
+        <v>33.07514882490723</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>UT5bq9li</t>
+          <t>4nxtRRYM</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45466.10416666666</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>los angeles fc</t>
+          <t>minnesota united</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>san jose earthquakes</t>
+          <t>austin fc</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -3389,85 +3389,85 @@
         <v>1671</v>
       </c>
       <c r="G40" t="n">
-        <v>1.36</v>
+        <v>1.73</v>
       </c>
       <c r="H40" t="n">
-        <v>5.25</v>
+        <v>4</v>
       </c>
       <c r="I40" t="n">
-        <v>7</v>
+        <v>4.33</v>
       </c>
       <c r="J40" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.54584017471928</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1782437745740498</v>
+        <v>0.2360758755660886</v>
       </c>
       <c r="L40" t="n">
-        <v>0.1336828309305373</v>
+        <v>0.2180839497146315</v>
       </c>
       <c r="M40" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.05898156429801493</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>0.6288124535672187</v>
+        <v>0.3723226691402557</v>
       </c>
       <c r="P40" t="n">
-        <v>0.3013673527911105</v>
+        <v>0.1948158673714422</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.06982019364167102</v>
+        <v>0.4328614634883022</v>
       </c>
       <c r="R40" t="n">
         <v>1</v>
       </c>
       <c r="S40" t="n">
-        <v>-0.05926094092819412</v>
+        <v>0.2147775137736708</v>
       </c>
       <c r="T40" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="U40" t="n">
-        <v>0.05926094092819412</v>
+        <v>0.2147775137736708</v>
       </c>
       <c r="V40" t="n">
-        <v>0.3711875464327813</v>
+        <v>0.4328614634883022</v>
       </c>
       <c r="W40" t="n">
-        <v>3</v>
+        <v>4.33</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y40" t="n">
-        <v>25.98312825029469</v>
+        <v>30.30030244418116</v>
       </c>
       <c r="Z40" t="n">
-        <v>25.98312825029469</v>
+        <v>30.30030244418116</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>Ma0gz0nH</t>
+          <t>IktpQolT</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45466.10416666666</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>portland timbers</t>
+          <t>nashville sc</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>vancouver whitecaps</t>
+          <t>new york city</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -3477,85 +3477,85 @@
         <v>1671</v>
       </c>
       <c r="G41" t="n">
-        <v>2.15</v>
+        <v>2.63</v>
       </c>
       <c r="H41" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="I41" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
       <c r="J41" t="n">
-        <v>0.439632042928325</v>
+        <v>0.3619297617627173</v>
       </c>
       <c r="K41" t="n">
-        <v>0.2554618627826753</v>
+        <v>0.2719643638388418</v>
       </c>
       <c r="L41" t="n">
-        <v>0.3049060942889996</v>
+        <v>0.3661058743984409</v>
       </c>
       <c r="M41" t="n">
-        <v>0.05796719450132803</v>
+        <v>0.05055780721179959</v>
       </c>
       <c r="N41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O41" t="n">
-        <v>0.5201066341798269</v>
+        <v>0.3328004140349778</v>
       </c>
       <c r="P41" t="n">
-        <v>0.4046451603515387</v>
+        <v>0.426784241468339</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.07524820546863475</v>
+        <v>0.2404153444966831</v>
       </c>
       <c r="R41" t="n">
         <v>1</v>
       </c>
       <c r="S41" t="n">
-        <v>0.08047459125150191</v>
+        <v>0.1548198776294972</v>
       </c>
       <c r="T41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>0.08047459125150191</v>
+        <v>0.1548198776294972</v>
       </c>
       <c r="V41" t="n">
-        <v>0.5201066341798269</v>
+        <v>0.426784241468339</v>
       </c>
       <c r="W41" t="n">
-        <v>2.15</v>
+        <v>3.5</v>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y41" t="n">
-        <v>36.40746439258788</v>
+        <v>29.87489690278373</v>
       </c>
       <c r="Z41" t="n">
-        <v>36.40746439258788</v>
+        <v>29.87489690278373</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>8K42rT3c</t>
+          <t>OWICL5dp</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45466.10416666666</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>seattle sounders</t>
+          <t>st  louis city</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>fc dallas</t>
+          <t>atlanta utd</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -3565,66 +3565,66 @@
         <v>1671</v>
       </c>
       <c r="G42" t="n">
-        <v>1.45</v>
+        <v>1.83</v>
       </c>
       <c r="H42" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="I42" t="n">
-        <v>7</v>
+        <v>3.7</v>
       </c>
       <c r="J42" t="n">
-        <v>0.6538661131292164</v>
+        <v>0.5180518051805181</v>
       </c>
       <c r="K42" t="n">
-        <v>0.210690192008303</v>
+        <v>0.2257225722572257</v>
       </c>
       <c r="L42" t="n">
-        <v>0.1354436948624805</v>
+        <v>0.2562256225622562</v>
       </c>
       <c r="M42" t="n">
-        <v>0.05473453749315826</v>
+        <v>0.05481359579720224</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>0.3745130758574692</v>
+        <v>0.2032595674696957</v>
       </c>
       <c r="P42" t="n">
-        <v>0.4403573203792</v>
+        <v>0.2226757413052</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.1851296037633309</v>
+        <v>0.5740646912251044</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
       </c>
       <c r="S42" t="n">
-        <v>0.229667128370897</v>
+        <v>0.3178390686628482</v>
       </c>
       <c r="T42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U42" t="n">
-        <v>0.229667128370897</v>
+        <v>0.3178390686628482</v>
       </c>
       <c r="V42" t="n">
-        <v>0.4403573203792</v>
+        <v>0.5740646912251044</v>
       </c>
       <c r="W42" t="n">
-        <v>4.5</v>
+        <v>3.7</v>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y42" t="n">
-        <v>30.825012426544</v>
+        <v>40.18452838575731</v>
       </c>
       <c r="Z42" t="n">
-        <v>30.825012426544</v>
+        <v>40.18452838575731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>